<commit_message>
Inclusão de colunas 'Interno Sistema'
</commit_message>
<xml_diff>
--- a/DICIONARIO DE DADOS.xlsx
+++ b/DICIONARIO DE DADOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0-Repositorios\sql-migracao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66C104B-F1EF-4874-92E6-8EFB8440DEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68A760C-E4E5-49A4-AF1C-8F49DFDCE718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="920" xr2:uid="{365E4779-0F30-4366-ADA5-894CEE121BCE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="920" firstSheet="1" activeTab="9" xr2:uid="{365E4779-0F30-4366-ADA5-894CEE121BCE}"/>
   </bookViews>
   <sheets>
     <sheet name="ALT CADASTRAIS" sheetId="12" r:id="rId1"/>
@@ -3754,7 +3754,13 @@
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6E7FD2C1-E480-4BFF-8921-408BA731D000}" name="CONTRATO" displayName="CONTRATO" ref="A1:E144" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:E144" xr:uid="{6E7FD2C1-E480-4BFF-8921-408BA731D000}"/>
+  <autoFilter ref="A1:E144" xr:uid="{6E7FD2C1-E480-4BFF-8921-408BA731D000}">
+    <filterColumn colId="3">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3C12D3CA-82E1-4D12-9D13-E5319871A469}" uniqueName="1" name="TM" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{05269625-8E6E-451A-95E7-F0B8439467BD}" uniqueName="2" name="F" queryTableFieldId="2" dataDxfId="7"/>
@@ -4448,7 +4454,7 @@
 alteração. Caso não seja informada, será gravada a atual.],</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4475,7 +4481,7 @@
 conversões para o Darwin.],</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>40</v>
       </c>
@@ -4748,7 +4754,7 @@
         <v>LEFT(CAST(PFUNC.CODSITUACAO AS VARCHAR), 1) AS [Situação:],</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -4767,7 +4773,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [1 – Ativo],</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -4786,7 +4792,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [2 – Afastado],</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>7</v>
       </c>
@@ -4805,7 +4811,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [3 – Rescindido no Mês],</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>7</v>
       </c>
@@ -4886,7 +4892,7 @@
         <v>LEFT(CAST(PFUNC.CODRECEBIMENTO AS VARCHAR), 1) AS [Tipo de Salário:],</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>7</v>
       </c>
@@ -4901,7 +4907,7 @@
         <v>[1 – Mensal]</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>7</v>
       </c>
@@ -4916,7 +4922,7 @@
         <v>[2 – Por Quinzena]</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -4931,7 +4937,7 @@
         <v>[3 – Por Semana]</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>7</v>
       </c>
@@ -4946,7 +4952,7 @@
         <v>[4 – Por Dia]</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>7</v>
       </c>
@@ -4961,7 +4967,7 @@
         <v>[5 – Por Hora]</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>7</v>
       </c>
@@ -4976,7 +4982,7 @@
         <v>[6 – Por Tarefa]</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>7</v>
       </c>
@@ -5115,7 +5121,7 @@
         <v>'' AS [Nível de Exposição a Agente Nocivo:],</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>7</v>
       </c>
@@ -5134,7 +5140,7 @@
         <v>'' AS [00 – Nunca esteve exposto],</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>7</v>
       </c>
@@ -5153,7 +5159,7 @@
         <v>'' AS [01 – Não exposto, mas já esteve],</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>7</v>
       </c>
@@ -5172,7 +5178,7 @@
         <v>'' AS [02 – Exposto com aposentadoria aos 15 anos],</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>7</v>
       </c>
@@ -5191,7 +5197,7 @@
         <v>'' AS [03 – Exposto com aposentadoria aos 20 anos],</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>7</v>
       </c>
@@ -5210,7 +5216,7 @@
         <v>'' AS [04 – Exposto com aposentadoria aos 25 anos],</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>7</v>
       </c>
@@ -5229,7 +5235,7 @@
         <v>'' AS [05 – Não exposto com mais de um vínculo],</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>7</v>
       </c>
@@ -5248,7 +5254,7 @@
         <v>'' AS [06 – Exposto c/aposentadoria 15 anos e mais de um vínculo],</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>7</v>
       </c>
@@ -5267,7 +5273,7 @@
         <v>'' AS [07 – Exposto c/aposentadoria 20 anos e mais de um vínculo],</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>7</v>
       </c>
@@ -5670,7 +5676,7 @@
         <v>2 AS [Tipo de Contrato],</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>7</v>
       </c>
@@ -5689,7 +5695,7 @@
         <v>'' AS [1 - Determinado],</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>7</v>
       </c>
@@ -5730,7 +5736,7 @@
         <v>'' AS [Motivo de Rescisão Darwin],</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>7</v>
       </c>
@@ -5745,7 +5751,7 @@
         <v>[001 – Demissão com Justa Causa]</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>7</v>
       </c>
@@ -5760,7 +5766,7 @@
         <v>[002 – Demissão Sem Justa Causa]</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>7</v>
       </c>
@@ -5775,7 +5781,7 @@
         <v>[003 – Pedido de Demissão Sem Justa Causa]</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>7</v>
       </c>
@@ -5790,7 +5796,7 @@
         <v>[005 – Rescisão Por Término de Contrato Prazo Determinado]</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>7</v>
       </c>
@@ -5805,7 +5811,7 @@
         <v>[006 – Resc. Ant. do Contr. Por Prazo Determinado p/Empregado]</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>7</v>
       </c>
@@ -5820,7 +5826,7 @@
         <v>[007 – Resc. Ant. do Contr. Por Prazo Determinado p/Empresa]</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>7</v>
       </c>
@@ -5835,7 +5841,7 @@
         <v>[008 – Rescisão p/Término de Contr. Temporário]</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>7</v>
       </c>
@@ -5850,7 +5856,7 @@
         <v>[009 – Rescisão por Dispensa Indireta]</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>7</v>
       </c>
@@ -5865,7 +5871,7 @@
         <v>[010 – Rescisão por Culpa Recíproca]</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>7</v>
       </c>
@@ -5880,7 +5886,7 @@
         <v>[011 – Transferência de Estab. c/Ônus p/Cedente]</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>7</v>
       </c>
@@ -5895,7 +5901,7 @@
         <v>[012 – Transferência de Estab. s/Ônus p/Cedente]</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>7</v>
       </c>
@@ -5910,7 +5916,7 @@
         <v>[013 – Mudança de Regime Trabalhista]</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
         <v>7</v>
       </c>
@@ -5925,7 +5931,7 @@
         <v>[014 – Reforma de Militar]</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>7</v>
       </c>
@@ -5940,7 +5946,7 @@
         <v>[015 – Demissão sem Justa Causa Empr. Doméstico]</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>7</v>
       </c>
@@ -5955,7 +5961,7 @@
         <v>[016 – Rescisão por Acordo Entre as Partes]</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>7</v>
       </c>
@@ -5970,7 +5976,7 @@
         <v>[017 – Desligamento p/Tranf. Outro Sistema]</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>7</v>
       </c>
@@ -5985,7 +5991,7 @@
         <v>[020 – Falecimento]</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>7</v>
       </c>
@@ -6000,7 +6006,7 @@
         <v>[021 – Falecimento Decorr. de Acidente do Trabalho]</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>7</v>
       </c>
@@ -6015,7 +6021,7 @@
         <v>[022 – Falecimento Decorr. de Doença Pr.]</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>7</v>
       </c>
@@ -6030,7 +6036,7 @@
         <v>[023 – Falecimento Decorr. de Acidente no Trajeto]</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>7</v>
       </c>
@@ -6045,7 +6051,7 @@
         <v>[030 – Aposentadoria por Tempo de Serviço]</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>7</v>
       </c>
@@ -6060,7 +6066,7 @@
         <v>[031 – Aposentadoria por Idade]</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
         <v>7</v>
       </c>
@@ -6075,7 +6081,7 @@
         <v>[032 – Aposentadoria por Invalidez]</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>7</v>
       </c>
@@ -6090,7 +6096,7 @@
         <v>[033 – Aposentadoria p/Invalidez Dec.Acid.Trab.]</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
         <v>7</v>
       </c>
@@ -6105,7 +6111,7 @@
         <v>[034 – Aposentadoria p/Invalidez Dec.Doença Pr.]</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>7</v>
       </c>
@@ -6120,7 +6126,7 @@
         <v>[035 - Aposentadoria Compulsória]</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
         <v>7</v>
       </c>
@@ -6135,7 +6141,7 @@
         <v>[036 - Aposentadoria Especial]</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>7</v>
       </c>
@@ -6150,7 +6156,7 @@
         <v>[037 - Termino de Contrato - Estagiário]</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>7</v>
       </c>
@@ -6165,7 +6171,7 @@
         <v>[040 - Posse em outro Cargo Inacumulável]</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>7</v>
       </c>
@@ -6180,7 +6186,7 @@
         <v>[041 - Rescisão determinada pela Justiça]</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>7</v>
       </c>
@@ -6195,7 +6201,7 @@
         <v>[043 - Rescisão por Nulidade do Contrato Trab.]</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>7</v>
       </c>
@@ -6210,7 +6216,7 @@
         <v>[044 - Exoneração Diretor Não Empreg. s/J Causa]</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>7</v>
       </c>
@@ -6225,7 +6231,7 @@
         <v>[045 - Término de Mandato do Diretor Não Empreg]</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>7</v>
       </c>
@@ -6240,7 +6246,7 @@
         <v>[046 - Exoneração a pedido de Diretor Não Empr.]</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>7</v>
       </c>
@@ -6255,7 +6261,7 @@
         <v>[047 - Exoneração Diretor Não Empreg. Culpa Rec]</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>7</v>
       </c>
@@ -6270,7 +6276,7 @@
         <v>[048 - Morte do Diretor Não Empregado]</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>7</v>
       </c>
@@ -6285,7 +6291,7 @@
         <v>[049 - Exoneração Diretor Não Empregado p/Falên]</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>7</v>
       </c>
@@ -6300,7 +6306,7 @@
         <v>[1401 - Aprendiz - Término de Contrato]</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>7</v>
       </c>
@@ -6315,7 +6321,7 @@
         <v>[1402 - Aprendiz - Implemento da Idade]</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>7</v>
       </c>
@@ -6330,7 +6336,7 @@
         <v>[1403 - Aprendiz - Desemp. Insuf. ou Inadaptação]</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>7</v>
       </c>
@@ -6345,7 +6351,7 @@
         <v>[1404 - Aprendiz - Falta Disciplinar Grave]</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>7</v>
       </c>
@@ -6360,7 +6366,7 @@
         <v>[1405 - Aprendiz - Ausência Injustific. à Escola]</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>7</v>
       </c>
@@ -6375,7 +6381,7 @@
         <v>[1406 - Aprendiz - A Pedido do Aprendiz]</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>7</v>
       </c>
@@ -6390,7 +6396,7 @@
         <v>[1407 - Aprendiz - Fechamento da Empresa]</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>7</v>
       </c>
@@ -6436,7 +6442,7 @@
         <v>LEFT(CAST(PFUNC.CODCATEGORIAESOCIAL AS VARCHAR), 8) AS [Vínculo Empregatício:],</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E99" t="s">
         <v>346</v>
       </c>
@@ -6449,7 +6455,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [001-CLT - Empregador Pessoa Jurídica, categoria e-Social 101 - Empregado],</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>7</v>
       </c>
@@ -6470,7 +6476,7 @@
 contratado pela CLT],</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>7</v>
       </c>
@@ -6489,7 +6495,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [002 -Aprendiz, categoria e-Social 103 - Empregado – Aprendiz],</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>7</v>
       </c>
@@ -6510,7 +6516,7 @@
 Contrato de trabalho intermitenteIntermitente,categoriae-Social111-Empregado-],</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>7</v>
       </c>
@@ -6529,7 +6535,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [004 -Estagiário, categoria e-Social 901 - Estagiário],</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>7</v>
       </c>
@@ -6548,7 +6554,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [006-TrabalhadorTemporário-Lei6.019,categoriae-Social106-],</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E105" t="s">
         <v>352</v>
       </c>
@@ -6561,7 +6567,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [Trabalhador Temporário - contrato nos termos da Lei 6.019/74],</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>7</v>
       </c>
@@ -6580,7 +6586,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [007-TrabalhadorTemporário-Lei9.601,categoriae-Social105-],</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
         <v>354</v>
       </c>
@@ -6593,7 +6599,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [Empregado – contrato a termo firmado nos termos da Lei 9601/98],</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
         <v>355</v>
       </c>
@@ -6606,7 +6612,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [008 - CLT - Prazo Determinado Fixo ou Obra Certa, categoria e-Social 101 -],</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>7</v>
       </c>
@@ -6627,7 +6633,7 @@
 ou indireta contratado pela CLT],</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
         <v>357</v>
       </c>
@@ -6640,7 +6646,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [009 - Trabalhador Rural - Empregador Pessoa Jurídica, categoria e-Social],</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>7</v>
       </c>
@@ -6661,7 +6667,7 @@
 direta ou indireta contratado pela CLT],</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>7</v>
       </c>
@@ -6684,7 +6690,7 @@
 ou indireta contratado pela CLT],</v>
       </c>
     </row>
-    <row r="113" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>7</v>
       </c>
@@ -6707,7 +6713,7 @@
 - sem acordo para antecipação mensal da multa rescisória do FGTSdeTrabalhoVerdeeAmarelosemMultaFGTSMensal,],</v>
       </c>
     </row>
-    <row r="114" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>7</v>
       </c>
@@ -6730,7 +6736,7 @@
 - com acordo para antecipação mensal da multa rescisória do FGTSdeTrabalhoVerdeeAmarelocomMultaFGTSMensal,],</v>
       </c>
     </row>
-    <row r="115" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>7</v>
       </c>
@@ -6751,7 +6757,7 @@
 Avulso PortuárioAvulsoPortuário, categoria e-Social 201 -Trabalhador],</v>
       </c>
     </row>
-    <row r="116" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>7</v>
       </c>
@@ -6772,7 +6778,7 @@
 Trabalhador Avulso Não PortuárioAvulsoNãoPortuário,categoriae-Social202-],</v>
       </c>
     </row>
-    <row r="117" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
         <v>7</v>
       </c>
@@ -6795,7 +6801,7 @@
 fiscal],</v>
       </c>
     </row>
-    <row r="118" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
         <v>7</v>
       </c>
@@ -6814,7 +6820,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [102 - Diretor com FGTS - Sócio, categoria do e-Social 723 - Contribuinte],</v>
       </c>
     </row>
-    <row r="119" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E119" t="s">
         <v>366</v>
       </c>
@@ -6827,7 +6833,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [individual – empresários, sócios e membro de conselho de administração ou],</v>
       </c>
     </row>
-    <row r="120" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E120" t="s">
         <v>367</v>
       </c>
@@ -6840,7 +6846,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [fiscal],</v>
       </c>
     </row>
-    <row r="121" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B121" t="s">
         <v>7</v>
       </c>
@@ -6859,7 +6865,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [103 - Diretor sem FGTS - Não Sócio, categoria e-social 722 - Contribuinte],</v>
       </c>
     </row>
-    <row r="122" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E122" t="s">
         <v>369</v>
       </c>
@@ -6872,7 +6878,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [individual – Diretor não empregado, sem FGTS],</v>
       </c>
     </row>
-    <row r="123" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
         <v>7</v>
       </c>
@@ -6891,7 +6897,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [104 - Diretor com FGTS - Não Sócio, categoria e-Social 721 - Contribuinte],</v>
       </c>
     </row>
-    <row r="124" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
         <v>371</v>
       </c>
@@ -6904,7 +6910,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [individual – Diretor não empregado, com FGTS],</v>
       </c>
     </row>
-    <row r="125" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B125" t="s">
         <v>7</v>
       </c>
@@ -6923,7 +6929,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [201-Autônomo,categoriae-Social701-Contribuinteindividual–],</v>
       </c>
     </row>
-    <row r="126" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E126" t="s">
         <v>373</v>
       </c>
@@ -6938,7 +6944,7 @@
 de contribuinte individual],</v>
       </c>
     </row>
-    <row r="127" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="E127" t="s">
         <v>374</v>
       </c>
@@ -6951,7 +6957,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [202-Freteiro-Carga,categoriae-Social712-Contribuinteindividual–],</v>
       </c>
     </row>
-    <row r="128" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
         <v>7</v>
       </c>
@@ -6970,7 +6976,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [Transportador autônomo de carga],</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
         <v>7</v>
       </c>
@@ -6991,7 +6997,7 @@
 – Transportador autônomo de passageiros],</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
         <v>7</v>
       </c>
@@ -7014,7 +7020,7 @@
 intermédio de Cooperativa de Trabalho],</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
         <v>7</v>
       </c>
@@ -7037,7 +7043,7 @@
 serviços por intermédio de cooperativa de trabalho],</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
         <v>7</v>
       </c>
@@ -7056,7 +7062,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [206 - Médico Residente, categoria e-Social 902 - Médico Residente],</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>7</v>
       </c>
@@ -7075,7 +7081,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [207 - MEI - Microempreendedor Individual, categoria e-Social 741 -Contribuinte individual - Microempreendedor Individual],</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>7</v>
       </c>
@@ -7094,7 +7100,7 @@
         <v>LEFT(CAST(. AS ), 0) AS [301 - Empregado(a) Doméstico(a), categoria e-Social 104 - Empregado-Doméstico],</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
         <v>7</v>
       </c>
@@ -7117,7 +7123,7 @@
 contratado pela CLT],</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
         <v>7</v>
       </c>
@@ -7138,7 +7144,7 @@
 uma das demais categorias de contribuinte individual],</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>7</v>
       </c>
@@ -7159,7 +7165,7 @@
 711 - Contribuinte individual – Transportador autônomo de passageiros],</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
         <v>7</v>
       </c>
@@ -7180,7 +7186,7 @@
 - Contribuinte individual – Transportador autônomo de carga],</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
         <v>7</v>
       </c>
@@ -7225,7 +7231,7 @@
         <v>'' AS [Tipo de Admissão para o eSocial],</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B141" t="s">
         <v>7</v>
       </c>
@@ -7236,7 +7242,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B142" t="s">
         <v>7</v>
       </c>
@@ -7247,7 +7253,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B143" t="s">
         <v>7</v>
       </c>
@@ -7258,7 +7264,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>7</v>
       </c>
@@ -14308,7 +14314,7 @@
         <v>[Código do Contrato]</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J2:J6" si="1">"'' AS "&amp;F3&amp;","</f>
+        <f t="shared" ref="J3:J6" si="1">"'' AS "&amp;F3&amp;","</f>
         <v>'' AS [Código do Contrato],</v>
       </c>
     </row>

</xml_diff>